<commit_message>
updated mermaids and calculator to stablish model for embebing
</commit_message>
<xml_diff>
--- a/docs/cost/llm-cost-calculator.xlsx
+++ b/docs/cost/llm-cost-calculator.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Supuestos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Calculo" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Escenarios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RAG" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +20,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);-"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0);-"/>
     <numFmt numFmtId="166" formatCode="$#,##0.000000;($#,##0.000000);-"/>
     <numFmt numFmtId="167" formatCode="$#,##0;($#,##0);-"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.0000"/>
+    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +91,13 @@
       <color rgb="001F4E78"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -143,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +184,16 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1766,4 +1786,769 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Calculadora RAG (modelo de embeddings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Modela el costo del modelo de EMBEDDINGS del RAG (indexar documentos + embeber la query) y los tokens extra de sintesis por los chunks recuperados. La generacion/sintesis sigue siendo el modelo planificador (Supuestos!B12, GPT-5.2). Precios representativos jun-2026: confirmar antes de presupuestar. Editar solo celdas amarillas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>1) Modelos de embeddings (comparacion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Input $/1M</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Dimensiones</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Max tokens entrada</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>MTEB retrieval (aprox)</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>Multilingue</t>
+        </is>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>text-embedding-3-small</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1536</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8191</v>
+      </c>
+      <c r="F6" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OpenAI pricing 2026; MTEB leaderboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>text-embedding-3-large</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3072</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8191</v>
+      </c>
+      <c r="F7" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>OpenAI pricing 2026; MTEB leaderboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>voyage-3-lite</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Voyage AI</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D8" t="n">
+        <v>512</v>
+      </c>
+      <c r="E8" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F8" t="n">
+        <v>64</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>voyageai.com pricing 2026 (Anthropic recomienda Voyage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>voyage-3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Voyage AI</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>67</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>voyageai.com pricing 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>embed v3 multilingual</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cohere</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E10" t="n">
+        <v>512</v>
+      </c>
+      <c r="F10" t="n">
+        <v>64</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>cohere.com pricing 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>gemini-embedding-001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3072</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2048</v>
+      </c>
+      <c r="F11" t="n">
+        <v>68</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ai.google.dev pricing 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>bge-m3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Workers AI / self-host</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1024</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8192</v>
+      </c>
+      <c r="F12" t="n">
+        <v>60</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Cloudflare Workers AI / infra (cross-cloud si se usa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>Fuentes (URLs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- OpenAI embeddings: https://openai.com/api/pricing/ ; MTEB: https://huggingface.co/spaces/mteb/leaderboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>- Voyage AI: https://www.voyageai.com/ (Anthropic recomienda Voyage; no tiene embeddings propios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Cohere Embed v3: https://cohere.com/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- Google gemini-embedding: https://ai.google.dev/gemini-api/docs/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>- Cloudflare Workers AI (bge-m3): https://developers.cloudflare.com/workers-ai/ (precio por neurona / infra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>2) Variables (editar celdas amarillas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Ingesta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>N documentos</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tokens promedio por documento</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>% documentos que cambian (reindex) por mes</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>Recuperacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>% interacciones que usan knowledge_lookup</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>top-k chunks recuperados</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tokens promedio por chunk</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tokens de query a embeber</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Modelo de embeddings seleccionado</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>text-embedding-3-small</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Modelo de sintesis (= Supuestos)</t>
+        </is>
+      </c>
+      <c r="B35">
+        <f>Supuestos!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>3) Calculo RAG (derivado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Precio embedding seleccionado $/1M</t>
+        </is>
+      </c>
+      <c r="B38" s="27">
+        <f>VLOOKUP(B34,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Precio input sintesis $/1M (chunks, no cacheable)</t>
+        </is>
+      </c>
+      <c r="B39" s="27">
+        <f>VLOOKUP(B35,Pricing!$A$5:$E$16,3,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Interacciones por mes (total)</t>
+        </is>
+      </c>
+      <c r="B40">
+        <f>Calculo!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Interacciones RAG por mes</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>B40*B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ingesta inicial one-time (USD)</t>
+        </is>
+      </c>
+      <c r="B43" s="30">
+        <f>B23*B24*B38/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Reindex por mes (USD)</t>
+        </is>
+      </c>
+      <c r="B44" s="30">
+        <f>B23*B25*B24*B38/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Query-embeddings por mes (USD)</t>
+        </is>
+      </c>
+      <c r="B45" s="30">
+        <f>B41*B31*B38/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Tokens extra de sintesis por mes (USD)</t>
+        </is>
+      </c>
+      <c r="B46" s="30">
+        <f>B41*B29*B30*B39/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>Total RAG incremental por mes (USD)</t>
+        </is>
+      </c>
+      <c r="B47" s="31">
+        <f>B44+B45+B46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Costo RAG incremental por interaccion-RAG (USD)</t>
+        </is>
+      </c>
+      <c r="B48" s="27">
+        <f>IF(B41=0,0,(B45+B46)/B41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="inlineStr">
+        <is>
+          <t>4) Comparacion: costo RAG/mes por modelo de embeddings (mismos supuestos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B51" s="26" t="inlineStr">
+        <is>
+          <t>Input $/1M</t>
+        </is>
+      </c>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>Total RAG/mes (USD)</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>Ingesta inicial (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <f>A6</f>
+        <v/>
+      </c>
+      <c r="B52" s="27">
+        <f>VLOOKUP($A52,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C52" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A52,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A52,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D52" s="30">
+        <f>B23*B24*VLOOKUP($A52,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <f>A7</f>
+        <v/>
+      </c>
+      <c r="B53" s="27">
+        <f>VLOOKUP($A53,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C53" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A53,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A53,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D53" s="30">
+        <f>B23*B24*VLOOKUP($A53,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <f>A8</f>
+        <v/>
+      </c>
+      <c r="B54" s="27">
+        <f>VLOOKUP($A54,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C54" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A54,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A54,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D54" s="30">
+        <f>B23*B24*VLOOKUP($A54,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <f>A9</f>
+        <v/>
+      </c>
+      <c r="B55" s="27">
+        <f>VLOOKUP($A55,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C55" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A55,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A55,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D55" s="30">
+        <f>B23*B24*VLOOKUP($A55,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <f>A10</f>
+        <v/>
+      </c>
+      <c r="B56" s="27">
+        <f>VLOOKUP($A56,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C56" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A56,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A56,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D56" s="30">
+        <f>B23*B24*VLOOKUP($A56,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <f>A11</f>
+        <v/>
+      </c>
+      <c r="B57" s="27">
+        <f>VLOOKUP($A57,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C57" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A57,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A57,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D57" s="30">
+        <f>B23*B24*VLOOKUP($A57,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <f>A12</f>
+        <v/>
+      </c>
+      <c r="B58" s="27">
+        <f>VLOOKUP($A58,$A$6:$H$12,3,0)</f>
+        <v/>
+      </c>
+      <c r="C58" s="30">
+        <f>(B23*B25*B24*VLOOKUP($A58,$A$6:$H$12,3,0)/1000000)+(B41*B31*VLOOKUP($A58,$A$6:$H$12,3,0)/1000000)+(B41*B29*B30*B39/1000000)</f>
+        <v/>
+      </c>
+      <c r="D58" s="30">
+        <f>B23*B24*VLOOKUP($A58,$A$6:$H$12,3,0)/1000000</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=$A$6:$A$12</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>